<commit_message>
latest update before average consumer redo
</commit_message>
<xml_diff>
--- a/Data/20240911_EP2024-4366_Modelling_Sectoral_Pathways_to_Net_Zero_Emissions_Section 2_Sectors_Charts (1).xlsx
+++ b/Data/20240911_EP2024-4366_Modelling_Sectoral_Pathways_to_Net_Zero_Emissions_Section 2_Sectors_Charts (1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unimelbcloud-my.sharepoint.com/personal/dominic_jones_grattaninstitute_edu_au/Documents/Energy/Analysis/analysis_cp_dj_2025/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{B58AD273-3445-485A-BB3D-F8F815F048DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{472EB7D9-68B4-4410-B154-4CCD0105B928}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="13_ncr:1_{B58AD273-3445-485A-BB3D-F8F815F048DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AF67A0D1-D3F6-44DD-8A94-2EB165626435}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="850" activeTab="6" xr2:uid="{234CDC66-7FDF-4433-8217-C560C895BCB5}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="850" activeTab="7" xr2:uid="{234CDC66-7FDF-4433-8217-C560C895BCB5}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="277">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="277">
   <si>
     <t>1)</t>
   </si>
@@ -3028,9 +3028,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>10</xdr:col>
-      <xdr:colOff>67585</xdr:colOff>
+      <xdr:colOff>64410</xdr:colOff>
       <xdr:row>26</xdr:row>
-      <xdr:rowOff>128217</xdr:rowOff>
+      <xdr:rowOff>125042</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -14187,7 +14187,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A019CDF-5B85-4F02-904A-B924C2EE5F79}">
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1" spans="1:16" ht="18.5">
@@ -14467,6 +14467,62 @@
       </c>
       <c r="P12">
         <v>433.81383113932901</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13">
+        <f>SUM(B8:B12)/3.6</f>
+        <v>248.59730424591368</v>
+      </c>
+      <c r="C13">
+        <f t="shared" ref="C13:G13" si="0">SUM(C8:C12)/3.6</f>
+        <v>283.51662269972405</v>
+      </c>
+      <c r="D13">
+        <f t="shared" si="0"/>
+        <v>320.13539401171187</v>
+      </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>368.37689369464204</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="0"/>
+        <v>411.56432902605735</v>
+      </c>
+      <c r="G13">
+        <f t="shared" si="0"/>
+        <v>455.58526902505184</v>
+      </c>
+      <c r="J13" t="s">
+        <v>5</v>
+      </c>
+      <c r="K13">
+        <f>SUM(K8:K12)/3.6</f>
+        <v>248.59730424591368</v>
+      </c>
+      <c r="L13">
+        <f t="shared" ref="L13" si="1">SUM(L8:L12)/3.6</f>
+        <v>288.16369018655263</v>
+      </c>
+      <c r="M13">
+        <f t="shared" ref="M13" si="2">SUM(M8:M12)/3.6</f>
+        <v>340.56060398130495</v>
+      </c>
+      <c r="N13">
+        <f t="shared" ref="N13" si="3">SUM(N8:N12)/3.6</f>
+        <v>440.86219555813557</v>
+      </c>
+      <c r="O13">
+        <f t="shared" ref="O13" si="4">SUM(O8:O12)/3.6</f>
+        <v>481.29284078255182</v>
+      </c>
+      <c r="P13">
+        <f t="shared" ref="P13" si="5">SUM(P8:P12)/3.6</f>
+        <v>513.3134086650997</v>
       </c>
     </row>
   </sheetData>
@@ -14692,12 +14748,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f7fbf89-e199-4f2b-84ea-127fbe818fcc">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="a3c73764-a836-4074-9b75-ad57c1810901" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -14924,20 +14982,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="6f7fbf89-e199-4f2b-84ea-127fbe818fcc">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="a3c73764-a836-4074-9b75-ad57c1810901" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{674A4055-6243-43ED-B379-C1B2C9CE390E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9ED4EFD4-C6C7-45DC-A422-06416C60CAF6}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="6f7fbf89-e199-4f2b-84ea-127fbe818fcc"/>
+    <ds:schemaRef ds:uri="a3c73764-a836-4074-9b75-ad57c1810901"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -14962,12 +15021,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9ED4EFD4-C6C7-45DC-A422-06416C60CAF6}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{674A4055-6243-43ED-B379-C1B2C9CE390E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="6f7fbf89-e199-4f2b-84ea-127fbe818fcc"/>
-    <ds:schemaRef ds:uri="a3c73764-a836-4074-9b75-ad57c1810901"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>